<commit_message>
latest modify import pob address
</commit_message>
<xml_diff>
--- a/public/member_template.xlsx
+++ b/public/member_template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>កាកបាទក្រហមកម្ពុជា</t>
   </si>
@@ -123,16 +123,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="[$-12000425]0"/>
     <numFmt numFmtId="179" formatCode="000"/>
-    <numFmt numFmtId="180" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,13 +194,6 @@
       <sz val="11"/>
       <name val="Khmer OS Battambang"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -675,148 +667,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -864,7 +856,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1434,8 +1426,8 @@
       <c r="L6" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="M6" s="17">
-        <v>45658</v>
+      <c r="M6" s="17" t="s">
+        <v>22</v>
       </c>
       <c r="N6" s="18" t="s">
         <v>23</v>
@@ -1443,7 +1435,9 @@
       <c r="O6" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="P6" s="10"/>
+      <c r="P6" s="10" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="7" ht="15" spans="1:6">
       <c r="A7" s="12" t="s">

</xml_diff>